<commit_message>
New os not supported Cortex
</commit_message>
<xml_diff>
--- a/src/Reporte_Discovery.xlsx
+++ b/src/Reporte_Discovery.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jesusarellano/Documents/TELCEL/AXONIUS/Desarrollo/src/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C73AE164-CC7E-E649-8609-99BEBB3E3F83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB2BA221-23C8-1B42-A40A-2E1BCBE59F10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20440" yWindow="-21200" windowWidth="30240" windowHeight="17120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1600" yWindow="1380" windowWidth="23820" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" r:id="rId1"/>
@@ -35,8 +35,8 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="66" r:id="rId11"/>
-    <pivotCache cacheId="67" r:id="rId12"/>
+    <pivotCache cacheId="16" r:id="rId11"/>
+    <pivotCache cacheId="17" r:id="rId12"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -1189,6 +1189,63 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="3" fontId="7" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="10" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="9" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="13" fillId="8" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1258,39 +1315,6 @@
     <xf numFmtId="0" fontId="7" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="6" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1356,30 +1380,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="7" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="13" fillId="10" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="13" fillId="9" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="13" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="13" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="13" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="13" fillId="8" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1510,7 +1510,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B0F87A7E-D022-2E4A-8DDE-C4E01F9C3F96}" name="PivotTable1" cacheId="67" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B0F87A7E-D022-2E4A-8DDE-C4E01F9C3F96}" name="PivotTable1" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B2:C5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField showAll="0"/>
@@ -1558,7 +1558,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E7C88826-A921-F241-A7D7-09240D889B29}" name="PivotTable2" cacheId="66" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{E7C88826-A921-F241-A7D7-09240D889B29}" name="PivotTable2" cacheId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B2:C5" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField showAll="0"/>
@@ -1898,7 +1898,7 @@
   <cols>
     <col min="1" max="3" width="12.5" style="24" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.1640625" style="24" customWidth="1"/>
-    <col min="5" max="5" width="17.5" style="24" customWidth="1"/>
+    <col min="5" max="5" width="18.6640625" style="24" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.1640625" style="31" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1911,186 +1911,186 @@
       <c r="F1" s="25"/>
     </row>
     <row r="2" spans="1:6" s="18" customFormat="1" ht="24">
-      <c r="A2" s="53"/>
-      <c r="B2" s="53"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="54"/>
+      <c r="A2" s="72"/>
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="73"/>
     </row>
     <row r="3" spans="1:6" ht="17.25" customHeight="1">
-      <c r="A3" s="73" t="s">
+      <c r="A3" s="92" t="s">
         <v>123</v>
       </c>
-      <c r="B3" s="74"/>
-      <c r="C3" s="74"/>
-      <c r="D3" s="74"/>
-      <c r="E3" s="75"/>
+      <c r="B3" s="93"/>
+      <c r="C3" s="93"/>
+      <c r="D3" s="93"/>
+      <c r="E3" s="94"/>
       <c r="F3" s="41">
         <v>7507</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="17.25" customHeight="1">
-      <c r="A4" s="55"/>
-      <c r="B4" s="63" t="s">
+      <c r="A4" s="74"/>
+      <c r="B4" s="82" t="s">
         <v>124</v>
       </c>
-      <c r="C4" s="64"/>
-      <c r="D4" s="64"/>
-      <c r="E4" s="65"/>
-      <c r="F4" s="109">
+      <c r="C4" s="83"/>
+      <c r="D4" s="83"/>
+      <c r="E4" s="84"/>
+      <c r="F4" s="53">
         <f>F5+F10+F13+F14</f>
         <v>3729</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="17.25" customHeight="1">
-      <c r="A5" s="56"/>
-      <c r="B5" s="58"/>
-      <c r="C5" s="69" t="s">
+      <c r="A5" s="75"/>
+      <c r="B5" s="77"/>
+      <c r="C5" s="88" t="s">
         <v>125</v>
       </c>
-      <c r="D5" s="70"/>
-      <c r="E5" s="70"/>
-      <c r="F5" s="111">
+      <c r="D5" s="89"/>
+      <c r="E5" s="89"/>
+      <c r="F5" s="55">
         <f>COUNTA(Inventario!B6:B1048576)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="17.25" customHeight="1">
-      <c r="A6" s="56"/>
-      <c r="B6" s="59"/>
-      <c r="C6" s="66"/>
-      <c r="D6" s="76" t="s">
+      <c r="A6" s="75"/>
+      <c r="B6" s="78"/>
+      <c r="C6" s="85"/>
+      <c r="D6" s="61" t="s">
         <v>126</v>
       </c>
-      <c r="E6" s="77"/>
-      <c r="F6" s="110">
+      <c r="E6" s="62"/>
+      <c r="F6" s="54">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="17.25" customHeight="1">
-      <c r="A7" s="56"/>
-      <c r="B7" s="59"/>
-      <c r="C7" s="67"/>
-      <c r="D7" s="76" t="s">
+      <c r="A7" s="75"/>
+      <c r="B7" s="78"/>
+      <c r="C7" s="86"/>
+      <c r="D7" s="61" t="s">
         <v>138</v>
       </c>
-      <c r="E7" s="77"/>
+      <c r="E7" s="62"/>
       <c r="F7" s="47">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="17.25" customHeight="1">
-      <c r="A8" s="56"/>
-      <c r="B8" s="59"/>
-      <c r="C8" s="67"/>
-      <c r="D8" s="58"/>
+      <c r="A8" s="75"/>
+      <c r="B8" s="78"/>
+      <c r="C8" s="86"/>
+      <c r="D8" s="77"/>
       <c r="E8" s="48" t="s">
         <v>139</v>
       </c>
-      <c r="F8" s="113">
+      <c r="F8" s="57">
         <f>F7-F9</f>
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="17.25" customHeight="1">
-      <c r="A9" s="56"/>
-      <c r="B9" s="59"/>
-      <c r="C9" s="68"/>
-      <c r="D9" s="60"/>
-      <c r="E9" s="112" t="s">
+      <c r="A9" s="75"/>
+      <c r="B9" s="78"/>
+      <c r="C9" s="87"/>
+      <c r="D9" s="79"/>
+      <c r="E9" s="56" t="s">
         <v>140</v>
       </c>
-      <c r="F9" s="114" cm="1">
-        <f t="array" ref="F9">SUM(COUNTIFS(Inventario!E6:E1048576, {"Oracle Solaris","Windows Server 2008 R2","Windows Server 2003 R2","SunOS 10","SunOS 11.1","SunOS 11.2","SunOS 11.3","IBM AIX 6.1","IBM AIX 7.1","IBM AIX 7.2","IBM AIX 5.3","SunOS 9","SunOS 11.4.23.69.3","SunOS 11.0","SunOS 11.4","SunOS 11.4.0.15.0"}, Inventario!F6:F1048576, "NO"))</f>
+      <c r="F9" s="58" cm="1">
+        <f t="array" ref="F9">SUM(COUNTIFS(Inventario!E6:E1048576, {"Oracle Solaris","Windows Server 2008 R2","Windows Server 2003 R2","SunOS 10","SunOS 11.1","SunOS 11.2","SunOS 11.3","IBM AIX 6.1","IBM AIX 7.1","IBM AIX 7.2","IBM AIX 5.3","SunOS 9","SunOS 11.4.23.69.3","SunOS 11.0","SunOS 11.4","SunOS 11.4.0.15.0","Linux Red Hat 5","Linux Red Hat 6","IBM AIX 6","HP HP-UX","Cisco ISE","Cisco IOS","VMWare ESXi 6","VMWare ESXi 6.5","VMWare ESXi 7.0.3","VMWare ESXi 8.0.3","Linux FreeBSD","Linux FreeBSD 6.2","Linux FreeBSD 7.1","Linux FreeBSD 8.2","Linux FreeBSD 9.2","Linux FreeBSD 11","Linux FreeBSD 12","Linux Photon OS (64-bit)","Linux Arch 7","Windows Server 2008","Windows Server 2003","Windows Server 2000","Linux Fedora","Linux Fedora 24","Linux openSUSE 12.5","Linux openSUSE 8.10"}, Inventario!F6:F1048576, "NO"))</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="17.25" customHeight="1">
-      <c r="A10" s="56"/>
-      <c r="B10" s="59"/>
-      <c r="C10" s="69" t="s">
+      <c r="A10" s="75"/>
+      <c r="B10" s="78"/>
+      <c r="C10" s="88" t="s">
         <v>127</v>
       </c>
-      <c r="D10" s="70"/>
-      <c r="E10" s="70"/>
-      <c r="F10" s="111">
+      <c r="D10" s="89"/>
+      <c r="E10" s="89"/>
+      <c r="F10" s="55">
         <f>COUNTA('Inventario - PC'!B6:B1048576)</f>
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="17.25" customHeight="1">
-      <c r="A11" s="56"/>
-      <c r="B11" s="59"/>
-      <c r="C11" s="61"/>
-      <c r="D11" s="71" t="s">
+      <c r="A11" s="75"/>
+      <c r="B11" s="78"/>
+      <c r="C11" s="80"/>
+      <c r="D11" s="90" t="s">
         <v>128</v>
       </c>
-      <c r="E11" s="72"/>
-      <c r="F11" s="115">
+      <c r="E11" s="91"/>
+      <c r="F11" s="59">
         <f>COUNTIF('Inventario - PC'!F6:F1048576,"SI")</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="17.25" customHeight="1">
-      <c r="A12" s="56"/>
-      <c r="B12" s="59"/>
-      <c r="C12" s="62"/>
-      <c r="D12" s="71" t="s">
+      <c r="A12" s="75"/>
+      <c r="B12" s="78"/>
+      <c r="C12" s="81"/>
+      <c r="D12" s="90" t="s">
         <v>129</v>
       </c>
-      <c r="E12" s="72"/>
-      <c r="F12" s="113">
+      <c r="E12" s="91"/>
+      <c r="F12" s="57">
         <f>COUNTIF('Inventario - PC'!F6:F1048576,"no")</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="17.25" customHeight="1">
-      <c r="A13" s="56"/>
-      <c r="B13" s="59"/>
-      <c r="C13" s="69" t="s">
+      <c r="A13" s="75"/>
+      <c r="B13" s="78"/>
+      <c r="C13" s="88" t="s">
         <v>130</v>
       </c>
-      <c r="D13" s="70"/>
-      <c r="E13" s="70"/>
-      <c r="F13" s="111">
+      <c r="D13" s="89"/>
+      <c r="E13" s="89"/>
+      <c r="F13" s="55">
         <v>3726</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="17.25" customHeight="1">
-      <c r="A14" s="56"/>
-      <c r="B14" s="60"/>
-      <c r="C14" s="69" t="s">
+      <c r="A14" s="75"/>
+      <c r="B14" s="79"/>
+      <c r="C14" s="88" t="s">
         <v>131</v>
       </c>
-      <c r="D14" s="70"/>
-      <c r="E14" s="70"/>
-      <c r="F14" s="111">
+      <c r="D14" s="89"/>
+      <c r="E14" s="89"/>
+      <c r="F14" s="55">
         <f>COUNTA('Inventario Identificados'!A5:A1048576)</f>
         <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="17.25" customHeight="1">
-      <c r="A15" s="56"/>
-      <c r="B15" s="63" t="s">
+      <c r="A15" s="75"/>
+      <c r="B15" s="82" t="s">
         <v>132</v>
       </c>
-      <c r="C15" s="64"/>
-      <c r="D15" s="64"/>
-      <c r="E15" s="65"/>
-      <c r="F15" s="116">
+      <c r="C15" s="83"/>
+      <c r="D15" s="83"/>
+      <c r="E15" s="84"/>
+      <c r="F15" s="60">
         <f>COUNTA('Inventario No Identificados'!A5:A1048576)</f>
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="17.25" customHeight="1">
-      <c r="A16" s="57"/>
-      <c r="B16" s="63" t="s">
+      <c r="A16" s="76"/>
+      <c r="B16" s="82" t="s">
         <v>133</v>
       </c>
-      <c r="C16" s="64"/>
-      <c r="D16" s="64"/>
-      <c r="E16" s="65"/>
+      <c r="C16" s="83"/>
+      <c r="D16" s="83"/>
+      <c r="E16" s="84"/>
       <c r="F16" s="42">
         <f>F3-F4-F15</f>
         <v>3777</v>
@@ -2113,62 +2113,53 @@
       <c r="F18" s="43"/>
     </row>
     <row r="19" spans="1:6" s="18" customFormat="1" ht="24">
-      <c r="A19" s="81" t="s">
+      <c r="A19" s="66" t="s">
         <v>134</v>
       </c>
-      <c r="B19" s="82"/>
-      <c r="C19" s="82"/>
-      <c r="D19" s="82"/>
-      <c r="E19" s="82"/>
-      <c r="F19" s="83"/>
+      <c r="B19" s="67"/>
+      <c r="C19" s="67"/>
+      <c r="D19" s="67"/>
+      <c r="E19" s="67"/>
+      <c r="F19" s="68"/>
     </row>
     <row r="20" spans="1:6" ht="17.25" customHeight="1">
-      <c r="A20" s="84" t="s">
+      <c r="A20" s="69" t="s">
         <v>135</v>
       </c>
-      <c r="B20" s="85"/>
-      <c r="C20" s="85"/>
-      <c r="D20" s="86"/>
-      <c r="E20" s="78" t="s">
+      <c r="B20" s="70"/>
+      <c r="C20" s="70"/>
+      <c r="D20" s="71"/>
+      <c r="E20" s="63" t="s">
         <v>141</v>
       </c>
-      <c r="F20" s="79"/>
+      <c r="F20" s="64"/>
     </row>
     <row r="21" spans="1:6" ht="17.25" customHeight="1">
-      <c r="A21" s="84" t="s">
+      <c r="A21" s="69" t="s">
         <v>136</v>
       </c>
-      <c r="B21" s="85"/>
-      <c r="C21" s="85"/>
-      <c r="D21" s="86"/>
-      <c r="E21" s="78" t="s">
+      <c r="B21" s="70"/>
+      <c r="C21" s="70"/>
+      <c r="D21" s="71"/>
+      <c r="E21" s="63" t="s">
         <v>141</v>
       </c>
-      <c r="F21" s="79"/>
+      <c r="F21" s="64"/>
     </row>
     <row r="22" spans="1:6" ht="17.25" customHeight="1">
-      <c r="A22" s="84" t="s">
+      <c r="A22" s="69" t="s">
         <v>137</v>
       </c>
-      <c r="B22" s="85"/>
-      <c r="C22" s="85"/>
-      <c r="D22" s="86"/>
-      <c r="E22" s="80" t="s">
+      <c r="B22" s="70"/>
+      <c r="C22" s="70"/>
+      <c r="D22" s="71"/>
+      <c r="E22" s="65" t="s">
         <v>142</v>
       </c>
-      <c r="F22" s="79"/>
+      <c r="F22" s="64"/>
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="A19:F19"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="A22:D22"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A4:A16"/>
     <mergeCell ref="B5:B14"/>
@@ -2185,6 +2176,15 @@
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="C5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A22:D22"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F5" location="Inventario!A1" display="Inventario!A1" xr:uid="{B80F5769-9041-D946-A663-3C05C393B9EF}"/>
@@ -2283,52 +2283,52 @@
       </c>
     </row>
     <row r="5" spans="2:7" ht="17.25" customHeight="1">
-      <c r="B5" s="100" t="s">
+      <c r="B5" s="108" t="s">
         <v>16</v>
       </c>
       <c r="C5" s="4"/>
       <c r="D5" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="103" t="s">
+      <c r="E5" s="111" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="106" t="s">
+      <c r="F5" s="114" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="103" t="s">
+      <c r="G5" s="111" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="6" spans="2:7" ht="17.25" customHeight="1">
-      <c r="B6" s="101"/>
+      <c r="B6" s="109"/>
       <c r="C6" s="4"/>
       <c r="D6" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="E6" s="104"/>
-      <c r="F6" s="107"/>
-      <c r="G6" s="104"/>
+      <c r="E6" s="112"/>
+      <c r="F6" s="115"/>
+      <c r="G6" s="112"/>
     </row>
     <row r="7" spans="2:7" ht="17.25" customHeight="1">
-      <c r="B7" s="101"/>
+      <c r="B7" s="109"/>
       <c r="C7" s="4"/>
       <c r="D7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="104"/>
-      <c r="F7" s="107"/>
-      <c r="G7" s="104"/>
+      <c r="E7" s="112"/>
+      <c r="F7" s="115"/>
+      <c r="G7" s="112"/>
     </row>
     <row r="8" spans="2:7" ht="17.25" customHeight="1">
-      <c r="B8" s="102"/>
+      <c r="B8" s="110"/>
       <c r="C8" s="4"/>
       <c r="D8" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="E8" s="105"/>
-      <c r="F8" s="108"/>
-      <c r="G8" s="105"/>
+      <c r="E8" s="113"/>
+      <c r="F8" s="116"/>
+      <c r="G8" s="113"/>
     </row>
     <row r="9" spans="2:7" ht="17.25" customHeight="1">
       <c r="B9" s="9" t="s">
@@ -2349,32 +2349,32 @@
       </c>
     </row>
     <row r="10" spans="2:7" ht="17.25" customHeight="1">
-      <c r="B10" s="100" t="s">
+      <c r="B10" s="108" t="s">
         <v>25</v>
       </c>
       <c r="C10" s="4"/>
       <c r="D10" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="103" t="s">
+      <c r="E10" s="111" t="s">
         <v>27</v>
       </c>
-      <c r="F10" s="106" t="s">
+      <c r="F10" s="114" t="s">
         <v>10</v>
       </c>
-      <c r="G10" s="103" t="s">
+      <c r="G10" s="111" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="11" spans="2:7" ht="17.25" customHeight="1">
-      <c r="B11" s="102"/>
+      <c r="B11" s="110"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E11" s="105"/>
-      <c r="F11" s="108"/>
-      <c r="G11" s="105"/>
+      <c r="E11" s="113"/>
+      <c r="F11" s="116"/>
+      <c r="G11" s="113"/>
     </row>
     <row r="12" spans="2:7" ht="17.25" customHeight="1">
       <c r="B12" s="3" t="s">
@@ -2681,7 +2681,7 @@
       </c>
     </row>
     <row r="30" spans="2:7" ht="17.25" customHeight="1">
-      <c r="B30" s="100" t="s">
+      <c r="B30" s="108" t="s">
         <v>16</v>
       </c>
       <c r="C30" s="4" t="s">
@@ -2690,35 +2690,35 @@
       <c r="D30" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="E30" s="103" t="s">
+      <c r="E30" s="111" t="s">
         <v>88</v>
       </c>
-      <c r="F30" s="106" t="s">
+      <c r="F30" s="114" t="s">
         <v>10</v>
       </c>
-      <c r="G30" s="103" t="s">
+      <c r="G30" s="111" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="31" spans="2:7" ht="17.25" customHeight="1">
-      <c r="B31" s="101"/>
+      <c r="B31" s="109"/>
       <c r="C31" s="4"/>
       <c r="D31" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="E31" s="104"/>
-      <c r="F31" s="107"/>
-      <c r="G31" s="104"/>
+      <c r="E31" s="112"/>
+      <c r="F31" s="115"/>
+      <c r="G31" s="112"/>
     </row>
     <row r="32" spans="2:7" ht="17.25" customHeight="1">
-      <c r="B32" s="102"/>
+      <c r="B32" s="110"/>
       <c r="C32" s="4"/>
       <c r="D32" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="E32" s="105"/>
-      <c r="F32" s="108"/>
-      <c r="G32" s="105"/>
+      <c r="E32" s="113"/>
+      <c r="F32" s="116"/>
+      <c r="G32" s="113"/>
     </row>
     <row r="33" spans="2:7" ht="17.25" customHeight="1">
       <c r="B33" s="3" t="s">
@@ -2818,47 +2818,47 @@
       <c r="D2" s="16"/>
     </row>
     <row r="3" spans="1:7" s="18" customFormat="1" ht="24">
-      <c r="A3" s="87" t="s">
+      <c r="A3" s="95" t="s">
         <v>121</v>
       </c>
-      <c r="B3" s="88"/>
-      <c r="C3" s="88"/>
-      <c r="D3" s="88"/>
-      <c r="E3" s="88"/>
-      <c r="F3" s="88"/>
-      <c r="G3" s="88"/>
+      <c r="B3" s="96"/>
+      <c r="C3" s="96"/>
+      <c r="D3" s="96"/>
+      <c r="E3" s="96"/>
+      <c r="F3" s="96"/>
+      <c r="G3" s="96"/>
     </row>
     <row r="4" spans="1:7" s="18" customFormat="1" ht="16" customHeight="1">
-      <c r="A4" s="89" t="s">
+      <c r="A4" s="97" t="s">
         <v>100</v>
       </c>
-      <c r="B4" s="91" t="s">
+      <c r="B4" s="99" t="s">
         <v>101</v>
       </c>
-      <c r="C4" s="91" t="s">
+      <c r="C4" s="99" t="s">
         <v>102</v>
       </c>
-      <c r="D4" s="91" t="s">
+      <c r="D4" s="99" t="s">
         <v>103</v>
       </c>
-      <c r="E4" s="91" t="s">
+      <c r="E4" s="99" t="s">
         <v>104</v>
       </c>
-      <c r="F4" s="91" t="s">
+      <c r="F4" s="99" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="91" t="s">
+      <c r="G4" s="99" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:7" s="18" customFormat="1" ht="17.25" customHeight="1">
-      <c r="A5" s="90"/>
-      <c r="B5" s="92"/>
-      <c r="C5" s="92"/>
-      <c r="D5" s="92"/>
-      <c r="E5" s="92"/>
-      <c r="F5" s="92"/>
-      <c r="G5" s="92"/>
+      <c r="A5" s="98"/>
+      <c r="B5" s="100"/>
+      <c r="C5" s="100"/>
+      <c r="D5" s="100"/>
+      <c r="E5" s="100"/>
+      <c r="F5" s="100"/>
+      <c r="G5" s="100"/>
     </row>
     <row r="6" spans="1:7" ht="17.25" customHeight="1">
       <c r="A6" s="19"/>
@@ -14207,14 +14207,14 @@
       <c r="F2" s="17"/>
     </row>
     <row r="3" spans="1:6" s="18" customFormat="1" ht="24">
-      <c r="A3" s="87" t="s">
+      <c r="A3" s="95" t="s">
         <v>120</v>
       </c>
-      <c r="B3" s="88"/>
-      <c r="C3" s="88"/>
-      <c r="D3" s="88"/>
-      <c r="E3" s="88"/>
-      <c r="F3" s="88"/>
+      <c r="B3" s="96"/>
+      <c r="C3" s="96"/>
+      <c r="D3" s="96"/>
+      <c r="E3" s="96"/>
+      <c r="F3" s="96"/>
     </row>
     <row r="4" spans="1:6" s="18" customFormat="1" ht="17">
       <c r="A4" s="44" t="s">
@@ -14307,64 +14307,64 @@
       <c r="J2" s="17"/>
     </row>
     <row r="3" spans="1:10" s="18" customFormat="1" ht="24">
-      <c r="A3" s="87" t="s">
+      <c r="A3" s="95" t="s">
         <v>114</v>
       </c>
-      <c r="B3" s="88"/>
-      <c r="C3" s="88"/>
-      <c r="D3" s="88"/>
-      <c r="E3" s="88"/>
-      <c r="F3" s="88"/>
-      <c r="G3" s="88"/>
-      <c r="H3" s="87"/>
-      <c r="I3" s="87"/>
-      <c r="J3" s="88"/>
+      <c r="B3" s="96"/>
+      <c r="C3" s="96"/>
+      <c r="D3" s="96"/>
+      <c r="E3" s="96"/>
+      <c r="F3" s="96"/>
+      <c r="G3" s="96"/>
+      <c r="H3" s="95"/>
+      <c r="I3" s="95"/>
+      <c r="J3" s="96"/>
     </row>
     <row r="4" spans="1:10" s="18" customFormat="1" ht="17.25" customHeight="1">
-      <c r="A4" s="89" t="s">
+      <c r="A4" s="97" t="s">
         <v>100</v>
       </c>
-      <c r="B4" s="91" t="s">
+      <c r="B4" s="99" t="s">
         <v>101</v>
       </c>
-      <c r="C4" s="91" t="s">
+      <c r="C4" s="99" t="s">
         <v>102</v>
       </c>
-      <c r="D4" s="91" t="s">
+      <c r="D4" s="99" t="s">
         <v>103</v>
       </c>
-      <c r="E4" s="91" t="s">
+      <c r="E4" s="99" t="s">
         <v>104</v>
       </c>
-      <c r="F4" s="91" t="s">
+      <c r="F4" s="99" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="91" t="s">
+      <c r="G4" s="99" t="s">
         <v>115</v>
       </c>
-      <c r="H4" s="93" t="s">
+      <c r="H4" s="101" t="s">
         <v>116</v>
       </c>
-      <c r="I4" s="93"/>
-      <c r="J4" s="91" t="s">
+      <c r="I4" s="101"/>
+      <c r="J4" s="99" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="17.25" customHeight="1">
-      <c r="A5" s="90"/>
-      <c r="B5" s="92"/>
-      <c r="C5" s="92"/>
-      <c r="D5" s="92"/>
-      <c r="E5" s="92"/>
-      <c r="F5" s="92"/>
-      <c r="G5" s="92"/>
+      <c r="A5" s="98"/>
+      <c r="B5" s="100"/>
+      <c r="C5" s="100"/>
+      <c r="D5" s="100"/>
+      <c r="E5" s="100"/>
+      <c r="F5" s="100"/>
+      <c r="G5" s="100"/>
       <c r="H5" s="46" t="s">
         <v>118</v>
       </c>
       <c r="I5" s="46" t="s">
         <v>119</v>
       </c>
-      <c r="J5" s="92"/>
+      <c r="J5" s="100"/>
     </row>
     <row r="6" spans="1:10" ht="18.75" customHeight="1">
       <c r="A6" s="19"/>
@@ -14433,55 +14433,55 @@
       <c r="H2" s="25"/>
     </row>
     <row r="3" spans="1:11" s="18" customFormat="1" ht="24">
-      <c r="A3" s="94" t="s">
+      <c r="A3" s="102" t="s">
         <v>110</v>
       </c>
-      <c r="B3" s="95"/>
-      <c r="C3" s="95"/>
-      <c r="D3" s="95"/>
-      <c r="E3" s="95"/>
-      <c r="F3" s="95"/>
-      <c r="G3" s="95"/>
-      <c r="H3" s="94"/>
+      <c r="B3" s="103"/>
+      <c r="C3" s="103"/>
+      <c r="D3" s="103"/>
+      <c r="E3" s="103"/>
+      <c r="F3" s="103"/>
+      <c r="G3" s="103"/>
+      <c r="H3" s="102"/>
       <c r="I3" s="27"/>
       <c r="J3" s="27"/>
       <c r="K3" s="27"/>
     </row>
     <row r="4" spans="1:11" ht="17.25" customHeight="1">
-      <c r="A4" s="96" t="s">
+      <c r="A4" s="104" t="s">
         <v>100</v>
       </c>
-      <c r="B4" s="97" t="s">
+      <c r="B4" s="105" t="s">
         <v>101</v>
       </c>
-      <c r="C4" s="98" t="s">
+      <c r="C4" s="106" t="s">
         <v>102</v>
       </c>
-      <c r="D4" s="91" t="s">
+      <c r="D4" s="99" t="s">
         <v>103</v>
       </c>
-      <c r="E4" s="91" t="s">
+      <c r="E4" s="99" t="s">
         <v>111</v>
       </c>
-      <c r="F4" s="99" t="s">
+      <c r="F4" s="107" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="91" t="s">
+      <c r="G4" s="99" t="s">
         <v>112</v>
       </c>
-      <c r="H4" s="96" t="s">
+      <c r="H4" s="104" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="17.25" customHeight="1">
-      <c r="A5" s="96"/>
-      <c r="B5" s="97"/>
-      <c r="C5" s="98"/>
-      <c r="D5" s="92"/>
-      <c r="E5" s="92"/>
-      <c r="F5" s="99"/>
-      <c r="G5" s="92"/>
-      <c r="H5" s="96"/>
+      <c r="A5" s="104"/>
+      <c r="B5" s="105"/>
+      <c r="C5" s="106"/>
+      <c r="D5" s="100"/>
+      <c r="E5" s="100"/>
+      <c r="F5" s="107"/>
+      <c r="G5" s="100"/>
+      <c r="H5" s="104"/>
     </row>
     <row r="6" spans="1:11" ht="17.25" customHeight="1">
       <c r="A6" s="28"/>
@@ -14540,13 +14540,13 @@
       <c r="E2" s="17"/>
     </row>
     <row r="3" spans="1:5" s="18" customFormat="1" ht="24">
-      <c r="A3" s="87" t="s">
+      <c r="A3" s="95" t="s">
         <v>109</v>
       </c>
-      <c r="B3" s="88"/>
-      <c r="C3" s="88"/>
-      <c r="D3" s="88"/>
-      <c r="E3" s="88"/>
+      <c r="B3" s="96"/>
+      <c r="C3" s="96"/>
+      <c r="D3" s="96"/>
+      <c r="E3" s="96"/>
     </row>
     <row r="4" spans="1:5" s="18" customFormat="1" ht="17.25" customHeight="1">
       <c r="A4" s="49" t="s">
@@ -14621,13 +14621,13 @@
       <c r="E2" s="17"/>
     </row>
     <row r="3" spans="1:5" s="18" customFormat="1" ht="24">
-      <c r="A3" s="87" t="s">
+      <c r="A3" s="95" t="s">
         <v>99</v>
       </c>
-      <c r="B3" s="88"/>
-      <c r="C3" s="88"/>
-      <c r="D3" s="88"/>
-      <c r="E3" s="88"/>
+      <c r="B3" s="96"/>
+      <c r="C3" s="96"/>
+      <c r="D3" s="96"/>
+      <c r="E3" s="96"/>
     </row>
     <row r="4" spans="1:5" s="18" customFormat="1" ht="17.25" customHeight="1">
       <c r="A4" s="49" t="s">

</xml_diff>